<commit_message>
updated reg healths with UC variables
</commit_message>
<xml_diff>
--- a/input/reg_health_mental.xlsx
+++ b/input/reg_health_mental.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\andy_local\SimPaths project files\SimPaths\input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DF70282-FA2F-4B0E-8AE0-ED4D25C04B44}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{14666344-F2DD-4E9A-BF67-BFFD8737BDC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Info" sheetId="7" r:id="rId1"/>
@@ -26,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="254" uniqueCount="57">
   <si>
     <t>REGRESSOR</t>
   </si>
@@ -195,12 +195,15 @@
   <si>
     <t>Cut12</t>
   </si>
+  <si>
+    <t>D_Econ_benefits_UC</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -208,6 +211,13 @@
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -234,18 +244,20 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1"/>
   </cellStyleXfs>
   <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="1"/>
     <xf numFmtId="2" fontId="1" fillId="0" borderId="1" xfId="1" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1" xr:uid="{AE6DDE21-AD95-48E3-8AE3-35962C4CCD8B}"/>
+    <cellStyle name="Normal 4" xfId="2" xr:uid="{AA6C3C34-B6E2-4319-AC53-4835D2087A0E}"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -3834,502 +3846,579 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19ED6DFE-C7BD-4842-98F1-709F3188C44C}">
-  <dimension ref="A1:M12"/>
+  <dimension ref="A1:N13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <cols>
-    <col min="1" max="16384" width="9.140625" style="1"/>
-  </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A1" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="2" t="s">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
         <v>32</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>33</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>34</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>35</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>36</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>37</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>38</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>39</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>40</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>41</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>42</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A2" s="2" t="s">
+      <c r="N1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>33</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B2">
         <v>1.5828236226510979</v>
       </c>
-      <c r="C2" s="1">
+      <c r="C2">
         <v>1.9800493678499301E-2</v>
       </c>
-      <c r="D2" s="1">
-        <v>0</v>
-      </c>
-      <c r="E2" s="1">
-        <v>0</v>
-      </c>
-      <c r="F2" s="1">
-        <v>0</v>
-      </c>
-      <c r="G2" s="1">
-        <v>0</v>
-      </c>
-      <c r="H2" s="1">
-        <v>0</v>
-      </c>
-      <c r="I2" s="1">
-        <v>0</v>
-      </c>
-      <c r="J2" s="1">
-        <v>0</v>
-      </c>
-      <c r="K2" s="1">
-        <v>0</v>
-      </c>
-      <c r="L2" s="1">
-        <v>0</v>
-      </c>
-      <c r="M2" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A3" s="2" t="s">
+      <c r="D2">
+        <v>0</v>
+      </c>
+      <c r="E2">
+        <v>0</v>
+      </c>
+      <c r="F2">
+        <v>0</v>
+      </c>
+      <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2">
+        <v>0</v>
+      </c>
+      <c r="I2">
+        <v>0</v>
+      </c>
+      <c r="J2">
+        <v>0</v>
+      </c>
+      <c r="K2">
+        <v>0</v>
+      </c>
+      <c r="L2">
+        <v>0</v>
+      </c>
+      <c r="M2">
+        <v>0</v>
+      </c>
+      <c r="N2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>34</v>
       </c>
-      <c r="B3" s="2">
+      <c r="B3">
         <v>-0.49475546789848474</v>
       </c>
-      <c r="C3" s="1">
-        <v>0</v>
-      </c>
-      <c r="D3" s="1">
+      <c r="C3">
+        <v>0</v>
+      </c>
+      <c r="D3">
         <v>1.3606842631112687E-2</v>
       </c>
-      <c r="E3" s="1">
-        <v>0</v>
-      </c>
-      <c r="F3" s="1">
-        <v>0</v>
-      </c>
-      <c r="G3" s="1">
-        <v>0</v>
-      </c>
-      <c r="H3" s="1">
-        <v>0</v>
-      </c>
-      <c r="I3" s="1">
-        <v>0</v>
-      </c>
-      <c r="J3" s="1">
-        <v>0</v>
-      </c>
-      <c r="K3" s="1">
-        <v>0</v>
-      </c>
-      <c r="L3" s="1">
-        <v>0</v>
-      </c>
-      <c r="M3" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A4" s="2" t="s">
+      <c r="E3">
+        <v>0</v>
+      </c>
+      <c r="F3">
+        <v>0</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <v>0</v>
+      </c>
+      <c r="I3">
+        <v>0</v>
+      </c>
+      <c r="J3">
+        <v>0</v>
+      </c>
+      <c r="K3">
+        <v>0</v>
+      </c>
+      <c r="L3">
+        <v>0</v>
+      </c>
+      <c r="M3">
+        <v>0</v>
+      </c>
+      <c r="N3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
         <v>35</v>
       </c>
-      <c r="B4" s="2">
+      <c r="B4">
         <v>0.81059663636884238</v>
       </c>
-      <c r="C4" s="1">
-        <v>0</v>
-      </c>
-      <c r="D4" s="1">
-        <v>0</v>
-      </c>
-      <c r="E4" s="1">
+      <c r="C4">
+        <v>0</v>
+      </c>
+      <c r="D4">
+        <v>0</v>
+      </c>
+      <c r="E4">
         <v>1.7330460787656893E-2</v>
       </c>
-      <c r="F4" s="1">
-        <v>0</v>
-      </c>
-      <c r="G4" s="1">
-        <v>0</v>
-      </c>
-      <c r="H4" s="1">
-        <v>0</v>
-      </c>
-      <c r="I4" s="1">
-        <v>0</v>
-      </c>
-      <c r="J4" s="1">
-        <v>0</v>
-      </c>
-      <c r="K4" s="1">
-        <v>0</v>
-      </c>
-      <c r="L4" s="1">
-        <v>0</v>
-      </c>
-      <c r="M4" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A5" s="2" t="s">
+      <c r="F4">
+        <v>0</v>
+      </c>
+      <c r="G4">
+        <v>0</v>
+      </c>
+      <c r="H4">
+        <v>0</v>
+      </c>
+      <c r="I4">
+        <v>0</v>
+      </c>
+      <c r="J4">
+        <v>0</v>
+      </c>
+      <c r="K4">
+        <v>0</v>
+      </c>
+      <c r="L4">
+        <v>0</v>
+      </c>
+      <c r="M4">
+        <v>0</v>
+      </c>
+      <c r="N4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>36</v>
       </c>
-      <c r="B5" s="2">
+      <c r="B5">
         <v>5.6687229266666368E-2</v>
       </c>
-      <c r="C5" s="1">
-        <v>0</v>
-      </c>
-      <c r="D5" s="1">
-        <v>0</v>
-      </c>
-      <c r="E5" s="1">
-        <v>0</v>
-      </c>
-      <c r="F5" s="1">
+      <c r="C5">
+        <v>0</v>
+      </c>
+      <c r="D5">
+        <v>0</v>
+      </c>
+      <c r="E5">
+        <v>0</v>
+      </c>
+      <c r="F5">
         <v>8.3808064742804944E-3</v>
       </c>
-      <c r="G5" s="1">
-        <v>0</v>
-      </c>
-      <c r="H5" s="1">
-        <v>0</v>
-      </c>
-      <c r="I5" s="1">
-        <v>0</v>
-      </c>
-      <c r="J5" s="1">
-        <v>0</v>
-      </c>
-      <c r="K5" s="1">
-        <v>0</v>
-      </c>
-      <c r="L5" s="1">
-        <v>0</v>
-      </c>
-      <c r="M5" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A6" s="2" t="s">
+      <c r="G5">
+        <v>0</v>
+      </c>
+      <c r="H5">
+        <v>0</v>
+      </c>
+      <c r="I5">
+        <v>0</v>
+      </c>
+      <c r="J5">
+        <v>0</v>
+      </c>
+      <c r="K5">
+        <v>0</v>
+      </c>
+      <c r="L5">
+        <v>0</v>
+      </c>
+      <c r="M5">
+        <v>0</v>
+      </c>
+      <c r="N5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
         <v>37</v>
       </c>
-      <c r="B6" s="2">
+      <c r="B6">
         <v>-3.0846646285374393E-2</v>
       </c>
-      <c r="C6" s="1">
-        <v>0</v>
-      </c>
-      <c r="D6" s="1">
-        <v>0</v>
-      </c>
-      <c r="E6" s="1">
-        <v>0</v>
-      </c>
-      <c r="F6" s="1">
-        <v>0</v>
-      </c>
-      <c r="G6" s="1">
+      <c r="C6">
+        <v>0</v>
+      </c>
+      <c r="D6">
+        <v>0</v>
+      </c>
+      <c r="E6">
+        <v>0</v>
+      </c>
+      <c r="F6">
+        <v>0</v>
+      </c>
+      <c r="G6">
         <v>8.7550195009294535E-3</v>
       </c>
-      <c r="H6" s="1">
-        <v>0</v>
-      </c>
-      <c r="I6" s="1">
-        <v>0</v>
-      </c>
-      <c r="J6" s="1">
-        <v>0</v>
-      </c>
-      <c r="K6" s="1">
-        <v>0</v>
-      </c>
-      <c r="L6" s="1">
-        <v>0</v>
-      </c>
-      <c r="M6" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A7" s="2" t="s">
+      <c r="H6">
+        <v>0</v>
+      </c>
+      <c r="I6">
+        <v>0</v>
+      </c>
+      <c r="J6">
+        <v>0</v>
+      </c>
+      <c r="K6">
+        <v>0</v>
+      </c>
+      <c r="L6">
+        <v>0</v>
+      </c>
+      <c r="M6">
+        <v>0</v>
+      </c>
+      <c r="N6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>38</v>
       </c>
-      <c r="B7" s="2">
+      <c r="B7">
         <v>8.2476617533024266E-2</v>
       </c>
-      <c r="C7" s="1">
-        <v>0</v>
-      </c>
-      <c r="D7" s="1">
-        <v>0</v>
-      </c>
-      <c r="E7" s="1">
-        <v>0</v>
-      </c>
-      <c r="F7" s="1">
-        <v>0</v>
-      </c>
-      <c r="G7" s="1">
-        <v>0</v>
-      </c>
-      <c r="H7" s="1">
+      <c r="C7">
+        <v>0</v>
+      </c>
+      <c r="D7">
+        <v>0</v>
+      </c>
+      <c r="E7">
+        <v>0</v>
+      </c>
+      <c r="F7">
+        <v>0</v>
+      </c>
+      <c r="G7">
+        <v>0</v>
+      </c>
+      <c r="H7">
         <v>1.4554938772697219E-2</v>
       </c>
-      <c r="I7" s="1">
-        <v>0</v>
-      </c>
-      <c r="J7" s="1">
-        <v>0</v>
-      </c>
-      <c r="K7" s="1">
-        <v>0</v>
-      </c>
-      <c r="L7" s="1">
-        <v>0</v>
-      </c>
-      <c r="M7" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A8" s="2" t="s">
+      <c r="I7">
+        <v>0</v>
+      </c>
+      <c r="J7">
+        <v>0</v>
+      </c>
+      <c r="K7">
+        <v>0</v>
+      </c>
+      <c r="L7">
+        <v>0</v>
+      </c>
+      <c r="M7">
+        <v>0</v>
+      </c>
+      <c r="N7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
         <v>39</v>
       </c>
-      <c r="B8" s="2">
+      <c r="B8">
         <v>9.081039491341078E-2</v>
       </c>
-      <c r="C8" s="1">
-        <v>0</v>
-      </c>
-      <c r="D8" s="1">
-        <v>0</v>
-      </c>
-      <c r="E8" s="1">
-        <v>0</v>
-      </c>
-      <c r="F8" s="1">
-        <v>0</v>
-      </c>
-      <c r="G8" s="1">
-        <v>0</v>
-      </c>
-      <c r="H8" s="1">
-        <v>0</v>
-      </c>
-      <c r="I8" s="1">
+      <c r="C8">
+        <v>0</v>
+      </c>
+      <c r="D8">
+        <v>0</v>
+      </c>
+      <c r="E8">
+        <v>0</v>
+      </c>
+      <c r="F8">
+        <v>0</v>
+      </c>
+      <c r="G8">
+        <v>0</v>
+      </c>
+      <c r="H8">
+        <v>0</v>
+      </c>
+      <c r="I8">
         <v>1.4399398628218501E-3</v>
       </c>
-      <c r="J8" s="1">
-        <v>0</v>
-      </c>
-      <c r="K8" s="1">
-        <v>0</v>
-      </c>
-      <c r="L8" s="1">
-        <v>0</v>
-      </c>
-      <c r="M8" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A9" s="2" t="s">
+      <c r="J8">
+        <v>0</v>
+      </c>
+      <c r="K8">
+        <v>0</v>
+      </c>
+      <c r="L8">
+        <v>0</v>
+      </c>
+      <c r="M8">
+        <v>0</v>
+      </c>
+      <c r="N8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
         <v>40</v>
       </c>
-      <c r="B9" s="2">
+      <c r="B9">
         <v>-2.7164707269627789E-2</v>
       </c>
-      <c r="C9" s="1">
-        <v>0</v>
-      </c>
-      <c r="D9" s="1">
-        <v>0</v>
-      </c>
-      <c r="E9" s="1">
-        <v>0</v>
-      </c>
-      <c r="F9" s="1">
-        <v>0</v>
-      </c>
-      <c r="G9" s="1">
-        <v>0</v>
-      </c>
-      <c r="H9" s="1">
-        <v>0</v>
-      </c>
-      <c r="I9" s="1">
-        <v>0</v>
-      </c>
-      <c r="J9" s="1">
+      <c r="C9">
+        <v>0</v>
+      </c>
+      <c r="D9">
+        <v>0</v>
+      </c>
+      <c r="E9">
+        <v>0</v>
+      </c>
+      <c r="F9">
+        <v>0</v>
+      </c>
+      <c r="G9">
+        <v>0</v>
+      </c>
+      <c r="H9">
+        <v>0</v>
+      </c>
+      <c r="I9">
+        <v>0</v>
+      </c>
+      <c r="J9">
         <v>1.4741260895766305E-3</v>
       </c>
-      <c r="K9" s="1">
-        <v>0</v>
-      </c>
-      <c r="L9" s="1">
-        <v>0</v>
-      </c>
-      <c r="M9" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A10" s="2" t="s">
+      <c r="K9">
+        <v>0</v>
+      </c>
+      <c r="L9">
+        <v>0</v>
+      </c>
+      <c r="M9">
+        <v>0</v>
+      </c>
+      <c r="N9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
         <v>41</v>
       </c>
-      <c r="B10" s="2">
+      <c r="B10">
         <v>2.61720445167601</v>
       </c>
-      <c r="C10" s="1">
-        <v>0</v>
-      </c>
-      <c r="D10" s="1">
-        <v>0</v>
-      </c>
-      <c r="E10" s="1">
-        <v>0</v>
-      </c>
-      <c r="F10" s="1">
-        <v>0</v>
-      </c>
-      <c r="G10" s="1">
-        <v>0</v>
-      </c>
-      <c r="H10" s="1">
-        <v>0</v>
-      </c>
-      <c r="I10" s="1">
-        <v>0</v>
-      </c>
-      <c r="J10" s="1">
-        <v>0</v>
-      </c>
-      <c r="K10" s="1">
+      <c r="C10">
+        <v>0</v>
+      </c>
+      <c r="D10">
+        <v>0</v>
+      </c>
+      <c r="E10">
+        <v>0</v>
+      </c>
+      <c r="F10">
+        <v>0</v>
+      </c>
+      <c r="G10">
+        <v>0</v>
+      </c>
+      <c r="H10">
+        <v>0</v>
+      </c>
+      <c r="I10">
+        <v>0</v>
+      </c>
+      <c r="J10">
+        <v>0</v>
+      </c>
+      <c r="K10">
         <v>8.895829539810246E-3</v>
       </c>
-      <c r="L10" s="1">
-        <v>0</v>
-      </c>
-      <c r="M10" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A11" s="2" t="s">
+      <c r="L10">
+        <v>0</v>
+      </c>
+      <c r="M10">
+        <v>0</v>
+      </c>
+      <c r="N10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
         <v>42</v>
       </c>
-      <c r="B11" s="2">
+      <c r="B11">
         <v>0.67301381744778732</v>
       </c>
-      <c r="C11" s="1">
-        <v>0</v>
-      </c>
-      <c r="D11" s="1">
-        <v>0</v>
-      </c>
-      <c r="E11" s="1">
-        <v>0</v>
-      </c>
-      <c r="F11" s="1">
-        <v>0</v>
-      </c>
-      <c r="G11" s="1">
-        <v>0</v>
-      </c>
-      <c r="H11" s="1">
-        <v>0</v>
-      </c>
-      <c r="I11" s="1">
-        <v>0</v>
-      </c>
-      <c r="J11" s="1">
-        <v>0</v>
-      </c>
-      <c r="K11" s="1">
-        <v>0</v>
-      </c>
-      <c r="L11" s="1">
+      <c r="C11">
+        <v>0</v>
+      </c>
+      <c r="D11">
+        <v>0</v>
+      </c>
+      <c r="E11">
+        <v>0</v>
+      </c>
+      <c r="F11">
+        <v>0</v>
+      </c>
+      <c r="G11">
+        <v>0</v>
+      </c>
+      <c r="H11">
+        <v>0</v>
+      </c>
+      <c r="I11">
+        <v>0</v>
+      </c>
+      <c r="J11">
+        <v>0</v>
+      </c>
+      <c r="K11">
+        <v>0</v>
+      </c>
+      <c r="L11">
         <v>5.5256660537722621E-3</v>
       </c>
-      <c r="M11" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A12" s="2" t="s">
+      <c r="M11">
+        <v>0</v>
+      </c>
+      <c r="N11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
         <v>43</v>
       </c>
-      <c r="B12" s="2">
+      <c r="B12">
         <v>0.36817061223167097</v>
       </c>
-      <c r="C12" s="1">
-        <v>0</v>
-      </c>
-      <c r="D12" s="1">
-        <v>0</v>
-      </c>
-      <c r="E12" s="1">
-        <v>0</v>
-      </c>
-      <c r="F12" s="1">
-        <v>0</v>
-      </c>
-      <c r="G12" s="1">
-        <v>0</v>
-      </c>
-      <c r="H12" s="1">
-        <v>0</v>
-      </c>
-      <c r="I12" s="1">
-        <v>0</v>
-      </c>
-      <c r="J12" s="1">
-        <v>0</v>
-      </c>
-      <c r="K12" s="1">
-        <v>0</v>
-      </c>
-      <c r="L12" s="1">
-        <v>0</v>
-      </c>
-      <c r="M12" s="1">
+      <c r="C12">
+        <v>0</v>
+      </c>
+      <c r="D12">
+        <v>0</v>
+      </c>
+      <c r="E12">
+        <v>0</v>
+      </c>
+      <c r="F12">
+        <v>0</v>
+      </c>
+      <c r="G12">
+        <v>0</v>
+      </c>
+      <c r="H12">
+        <v>0</v>
+      </c>
+      <c r="I12">
+        <v>0</v>
+      </c>
+      <c r="J12">
+        <v>0</v>
+      </c>
+      <c r="K12">
+        <v>0</v>
+      </c>
+      <c r="L12">
+        <v>0</v>
+      </c>
+      <c r="M12">
         <v>5.9131496057040576E-3</v>
+      </c>
+      <c r="N12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>56</v>
+      </c>
+      <c r="B13">
+        <v>0.312</v>
+      </c>
+      <c r="C13">
+        <v>0</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+      <c r="E13">
+        <v>0</v>
+      </c>
+      <c r="F13">
+        <v>0</v>
+      </c>
+      <c r="G13">
+        <v>0</v>
+      </c>
+      <c r="H13">
+        <v>0</v>
+      </c>
+      <c r="I13">
+        <v>0</v>
+      </c>
+      <c r="J13">
+        <v>0</v>
+      </c>
+      <c r="K13">
+        <v>0</v>
+      </c>
+      <c r="L13">
+        <v>0</v>
+      </c>
+      <c r="M13">
+        <v>0</v>
+      </c>
+      <c r="N13">
+        <v>2.3408999999999999E-2</v>
       </c>
     </row>
   </sheetData>
@@ -4339,13 +4428,13 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A93277EA-A3FA-4F87-A840-095FA0D38FE2}">
-  <dimension ref="A1:M12"/>
+  <dimension ref="A1:N13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -4385,8 +4474,11 @@
       <c r="M1" s="1" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>33</v>
       </c>
@@ -4426,8 +4518,11 @@
       <c r="M2" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>34</v>
       </c>
@@ -4467,8 +4562,11 @@
       <c r="M3" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>35</v>
       </c>
@@ -4508,8 +4606,11 @@
       <c r="M4" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>36</v>
       </c>
@@ -4549,8 +4650,11 @@
       <c r="M5" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>37</v>
       </c>
@@ -4590,8 +4694,11 @@
       <c r="M6" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>38</v>
       </c>
@@ -4631,8 +4738,11 @@
       <c r="M7" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>39</v>
       </c>
@@ -4672,8 +4782,11 @@
       <c r="M8" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>40</v>
       </c>
@@ -4713,8 +4826,11 @@
       <c r="M9" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>41</v>
       </c>
@@ -4754,8 +4870,11 @@
       <c r="M10" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>42</v>
       </c>
@@ -4795,8 +4914,11 @@
       <c r="M11" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>43</v>
       </c>
@@ -4835,6 +4957,53 @@
       </c>
       <c r="M12" s="1">
         <v>5.5863387314687334E-3</v>
+      </c>
+      <c r="N12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>56</v>
+      </c>
+      <c r="B13">
+        <v>0.312</v>
+      </c>
+      <c r="C13">
+        <v>0</v>
+      </c>
+      <c r="D13">
+        <v>0</v>
+      </c>
+      <c r="E13">
+        <v>0</v>
+      </c>
+      <c r="F13">
+        <v>0</v>
+      </c>
+      <c r="G13">
+        <v>0</v>
+      </c>
+      <c r="H13">
+        <v>0</v>
+      </c>
+      <c r="I13">
+        <v>0</v>
+      </c>
+      <c r="J13">
+        <v>0</v>
+      </c>
+      <c r="K13">
+        <v>0</v>
+      </c>
+      <c r="L13">
+        <v>0</v>
+      </c>
+      <c r="M13">
+        <v>0</v>
+      </c>
+      <c r="N13">
+        <v>2.3408999999999999E-2</v>
       </c>
     </row>
   </sheetData>
@@ -10619,13 +10788,13 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{01CE1170-73A3-4064-A59A-E2A113C17F8D}">
-  <dimension ref="A1:M12"/>
+  <dimension ref="A1:N13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -10665,8 +10834,11 @@
       <c r="M1" s="1" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>33</v>
       </c>
@@ -10706,8 +10878,11 @@
       <c r="M2" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>34</v>
       </c>
@@ -10747,8 +10922,11 @@
       <c r="M3" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>35</v>
       </c>
@@ -10788,8 +10966,11 @@
       <c r="M4" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>36</v>
       </c>
@@ -10829,8 +11010,11 @@
       <c r="M5" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>37</v>
       </c>
@@ -10870,8 +11054,11 @@
       <c r="M6" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>38</v>
       </c>
@@ -10911,8 +11098,11 @@
       <c r="M7" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>39</v>
       </c>
@@ -10952,8 +11142,11 @@
       <c r="M8" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>40</v>
       </c>
@@ -10993,8 +11186,11 @@
       <c r="M9" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>41</v>
       </c>
@@ -11034,8 +11230,11 @@
       <c r="M10" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>42</v>
       </c>
@@ -11075,8 +11274,11 @@
       <c r="M11" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>43</v>
       </c>
@@ -11115,6 +11317,53 @@
       </c>
       <c r="M12" s="1">
         <v>1.3204931675790993E-3</v>
+      </c>
+      <c r="N12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B13" s="1">
+        <v>0.78100000000000003</v>
+      </c>
+      <c r="C13" s="1">
+        <v>0</v>
+      </c>
+      <c r="D13" s="1">
+        <v>0</v>
+      </c>
+      <c r="E13" s="1">
+        <v>0</v>
+      </c>
+      <c r="F13" s="1">
+        <v>0</v>
+      </c>
+      <c r="G13" s="1">
+        <v>0</v>
+      </c>
+      <c r="H13" s="1">
+        <v>0</v>
+      </c>
+      <c r="I13" s="1">
+        <v>0</v>
+      </c>
+      <c r="J13" s="1">
+        <v>0</v>
+      </c>
+      <c r="K13" s="1">
+        <v>0</v>
+      </c>
+      <c r="L13" s="1">
+        <v>0</v>
+      </c>
+      <c r="M13" s="1">
+        <v>0</v>
+      </c>
+      <c r="N13" s="1">
+        <v>7.0755999999999999E-2</v>
       </c>
     </row>
   </sheetData>
@@ -11124,13 +11373,13 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C98EB7F6-69F5-4701-8609-C8F5A0E52064}">
-  <dimension ref="A1:M12"/>
+  <dimension ref="A1:N13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -11170,8 +11419,11 @@
       <c r="M1" s="1" t="s">
         <v>43</v>
       </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N1" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>33</v>
       </c>
@@ -11211,8 +11463,11 @@
       <c r="M2" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
         <v>34</v>
       </c>
@@ -11252,8 +11507,11 @@
       <c r="M3" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
         <v>35</v>
       </c>
@@ -11293,8 +11551,11 @@
       <c r="M4" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N4">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
         <v>36</v>
       </c>
@@ -11334,8 +11595,11 @@
       <c r="M5" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>37</v>
       </c>
@@ -11375,8 +11639,11 @@
       <c r="M6" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N6">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>38</v>
       </c>
@@ -11416,8 +11683,11 @@
       <c r="M7" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N7">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>39</v>
       </c>
@@ -11457,8 +11727,11 @@
       <c r="M8" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N8">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>40</v>
       </c>
@@ -11498,8 +11771,11 @@
       <c r="M9" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N9">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>41</v>
       </c>
@@ -11539,8 +11815,11 @@
       <c r="M10" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="11" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A11" s="2" t="s">
         <v>42</v>
       </c>
@@ -11580,8 +11859,11 @@
       <c r="M11" s="1">
         <v>0</v>
       </c>
-    </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="N11">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
         <v>43</v>
       </c>
@@ -11620,6 +11902,53 @@
       </c>
       <c r="M12" s="1">
         <v>1.2537189849700075E-3</v>
+      </c>
+      <c r="N12">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>56</v>
+      </c>
+      <c r="B13" s="1">
+        <v>0.78100000000000003</v>
+      </c>
+      <c r="C13" s="1">
+        <v>0</v>
+      </c>
+      <c r="D13" s="1">
+        <v>0</v>
+      </c>
+      <c r="E13" s="1">
+        <v>0</v>
+      </c>
+      <c r="F13" s="1">
+        <v>0</v>
+      </c>
+      <c r="G13" s="1">
+        <v>0</v>
+      </c>
+      <c r="H13" s="1">
+        <v>0</v>
+      </c>
+      <c r="I13" s="1">
+        <v>0</v>
+      </c>
+      <c r="J13" s="1">
+        <v>0</v>
+      </c>
+      <c r="K13" s="1">
+        <v>0</v>
+      </c>
+      <c r="L13" s="1">
+        <v>0</v>
+      </c>
+      <c r="M13" s="1">
+        <v>0</v>
+      </c>
+      <c r="N13" s="1">
+        <v>7.0755999999999999E-2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>